<commit_message>
stb expanded sequential explanations
</commit_message>
<xml_diff>
--- a/inst/app/metadata/stettehbaah_2024-08-16.xlsx
+++ b/inst/app/metadata/stettehbaah_2024-08-16.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/zprinsloo_worldbank_org/Documents/innovation_hub/InnovationHubDashboard/inst/app/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_6D68FDCE8F79A89360642C52EAAAD23310C181F4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{924F6C67-2211-4544-B55B-F11CFAEA1F12}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_6D68FDCE8F79A89360642C52EAAAD23310C181F4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{146F2A14-2170-4334-86CD-DF32A2FEF28D}"/>
   <bookViews>
-    <workbookView xWindow="26370" yWindow="750" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53880" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -93,7 +93,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss\ \U\T\C"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,6 +105,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -127,17 +135,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -441,12 +452,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="20.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="20.7265625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -481,7 +492,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -491,7 +502,7 @@
       <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E2" s="2">
@@ -517,6 +528,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{9BF06403-58DC-40FE-A2F8-7F5363678FE6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter>&amp;R_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Official Use Only</oddFooter>

</xml_diff>